<commit_message>
fix: handle show full info PL142
</commit_message>
<xml_diff>
--- a/public/templates/vat-annex-pl142-reduce8.xlsx
+++ b/public/templates/vat-annex-pl142-reduce8.xlsx
@@ -6043,7 +6043,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="336"/>
     </row>
-    <row r="20" s="84" customFormat="1" ht="16.5" customHeight="1" spans="1:15">
+    <row r="20" s="84" customFormat="1" spans="1:15">
       <c r="A20" s="91"/>
       <c r="B20" s="308" t="s">
         <v>52</v>
@@ -6259,7 +6259,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="336"/>
     </row>
-    <row r="30" s="84" customFormat="1" ht="16.5" customHeight="1" spans="1:15">
+    <row r="30" s="84" customFormat="1" spans="1:15">
       <c r="A30" s="91"/>
       <c r="B30" s="308" t="s">
         <v>52</v>

</xml_diff>